<commit_message>
new .ttl from Google sheet has been generated
</commit_message>
<xml_diff>
--- a/vocabulary.xlsx
+++ b/vocabulary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ460"/>
+  <dimension ref="A1:AZ461"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32926,6 +32926,72 @@
       <c r="AY460" t="inlineStr"/>
       <c r="AZ460" t="inlineStr"/>
     </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>vocab:1441</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>my test</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr"/>
+      <c r="D461" t="inlineStr"/>
+      <c r="E461" t="inlineStr"/>
+      <c r="F461" t="inlineStr"/>
+      <c r="G461" t="inlineStr"/>
+      <c r="H461" t="inlineStr"/>
+      <c r="I461" t="inlineStr"/>
+      <c r="J461" t="inlineStr"/>
+      <c r="K461" t="inlineStr"/>
+      <c r="L461" t="inlineStr"/>
+      <c r="M461" t="inlineStr"/>
+      <c r="N461" t="inlineStr"/>
+      <c r="O461" t="inlineStr"/>
+      <c r="P461" t="inlineStr"/>
+      <c r="Q461" t="inlineStr"/>
+      <c r="R461" t="inlineStr"/>
+      <c r="S461" t="inlineStr"/>
+      <c r="T461" t="inlineStr"/>
+      <c r="U461" t="inlineStr"/>
+      <c r="V461" t="inlineStr"/>
+      <c r="W461" t="inlineStr"/>
+      <c r="X461" t="inlineStr"/>
+      <c r="Y461" t="inlineStr">
+        <is>
+          <t>2025-06-05</t>
+        </is>
+      </c>
+      <c r="Z461" t="inlineStr"/>
+      <c r="AA461" t="inlineStr"/>
+      <c r="AB461" t="inlineStr"/>
+      <c r="AC461" t="inlineStr"/>
+      <c r="AD461" t="inlineStr"/>
+      <c r="AE461" t="inlineStr"/>
+      <c r="AF461" t="inlineStr"/>
+      <c r="AG461" t="inlineStr"/>
+      <c r="AH461" t="inlineStr"/>
+      <c r="AI461" t="inlineStr"/>
+      <c r="AJ461" t="inlineStr"/>
+      <c r="AK461" t="inlineStr"/>
+      <c r="AL461" t="inlineStr"/>
+      <c r="AM461" t="inlineStr"/>
+      <c r="AN461" t="inlineStr"/>
+      <c r="AO461" t="inlineStr"/>
+      <c r="AP461" t="inlineStr"/>
+      <c r="AQ461" t="inlineStr"/>
+      <c r="AR461" t="inlineStr"/>
+      <c r="AS461" t="inlineStr"/>
+      <c r="AT461" t="inlineStr"/>
+      <c r="AU461" t="inlineStr"/>
+      <c r="AV461" t="inlineStr"/>
+      <c r="AW461" t="inlineStr"/>
+      <c r="AX461" t="inlineStr"/>
+      <c r="AY461" t="inlineStr"/>
+      <c r="AZ461" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>